<commit_message>
add details for version update
</commit_message>
<xml_diff>
--- a/docs/Project_Planning/overall.xlsx
+++ b/docs/Project_Planning/overall.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="F:\Git_doc\Real-Time-Embedded-Programming\docs\Project_Planning\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{57544E11-D6E5-43B9-B529-6BD912D183EA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C4F57F2B-864A-4871-A09E-B7DFF2FDE5CA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="15500" tabRatio="992" activeTab="8" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -22,6 +22,7 @@
     <sheet name="开发log" sheetId="11" r:id="rId7"/>
     <sheet name="data" sheetId="13" r:id="rId8"/>
     <sheet name="线程管理_0409" sheetId="14" r:id="rId9"/>
+    <sheet name="线程管理_0409 _eng" sheetId="15" r:id="rId10"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -41,7 +42,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="231" uniqueCount="209">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="333" uniqueCount="235">
   <si>
     <t>Motion学习方面如何配置？</t>
   </si>
@@ -730,6 +731,110 @@
   </si>
   <si>
     <t>_synthesisThread</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>Main Loop (Pseudo Thread)</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>Microphone Capture Thread</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>Triggered via play(), processes data in the queue into playable audio data, and pushes it to the playback thread for playback</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>Processing function: synthesisTask()</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>Input queue: _textQueue</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>Output queue: _dataQueue</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>Triggered by queue data, processes the data and buffers the processed data to the internal speaker unit for playback</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>Input queue: _dataQueue</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>Output: internal PCM processing</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>Triggered by queue data, passes the queued data to executeMotion() for processing</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>Input queue: MotionQueue</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>Triggered by queue data, application-level task processing thread</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>Input queue: camera_queue</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>Thread-triggered callback, returns current frame</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>Callback trigger: onFrame()</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>Started directly during construction</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>Started by calling open() during construction</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>At start, a frame transmission pipeline is configured, and a callback is triggered when a frame is detected</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>During destruction, both the cap transmission and frame capture threads are stopped</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>Submodules are automatically destroyed when RobotSystem is destructed</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>module</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>thread name</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>file</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>star</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>stop</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>thread core</t>
     <phoneticPr fontId="2" type="noConversion"/>
   </si>
 </sst>
@@ -20740,7 +20845,7 @@
                 <a:schemeClr val="tx1"/>
               </a:solidFill>
             </a:rPr>
-            <a:t>CogniArm  V1.0</a:t>
+            <a:t>CogniArm  V2.0</a:t>
           </a:r>
           <a:endParaRPr lang="zh-CN" altLang="en-US" sz="2000">
             <a:solidFill>
@@ -21180,6 +21285,432 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{30A9DC4A-0CC4-4407-A248-561200CE148C}">
+  <dimension ref="B2:AB52"/>
+  <sheetFormatPr defaultColWidth="8.7265625" defaultRowHeight="14" x14ac:dyDescent="0.25"/>
+  <sheetData>
+    <row r="2" spans="2:28" x14ac:dyDescent="0.25">
+      <c r="B2" s="3" t="s">
+        <v>229</v>
+      </c>
+      <c r="F2" s="3" t="s">
+        <v>230</v>
+      </c>
+      <c r="H2" s="3" t="s">
+        <v>231</v>
+      </c>
+      <c r="L2" s="3" t="s">
+        <v>232</v>
+      </c>
+      <c r="T2" s="3" t="s">
+        <v>233</v>
+      </c>
+      <c r="Z2" s="3" t="s">
+        <v>234</v>
+      </c>
+    </row>
+    <row r="3" spans="2:28" x14ac:dyDescent="0.25">
+      <c r="B3" s="4" t="s">
+        <v>133</v>
+      </c>
+      <c r="F3" t="s">
+        <v>134</v>
+      </c>
+    </row>
+    <row r="4" spans="2:28" x14ac:dyDescent="0.25">
+      <c r="B4" s="3" t="s">
+        <v>209</v>
+      </c>
+    </row>
+    <row r="6" spans="2:28" x14ac:dyDescent="0.25">
+      <c r="B6" s="4" t="s">
+        <v>135</v>
+      </c>
+      <c r="F6" t="s">
+        <v>136</v>
+      </c>
+      <c r="H6" t="s">
+        <v>137</v>
+      </c>
+      <c r="L6" t="s">
+        <v>138</v>
+      </c>
+      <c r="T6" t="s">
+        <v>139</v>
+      </c>
+      <c r="Z6">
+        <v>3</v>
+      </c>
+      <c r="AB6" s="3" t="s">
+        <v>164</v>
+      </c>
+    </row>
+    <row r="7" spans="2:28" x14ac:dyDescent="0.25">
+      <c r="B7" s="3" t="s">
+        <v>210</v>
+      </c>
+      <c r="L7" t="s">
+        <v>140</v>
+      </c>
+      <c r="T7" t="s">
+        <v>141</v>
+      </c>
+    </row>
+    <row r="8" spans="2:28" x14ac:dyDescent="0.25">
+      <c r="L8" t="s">
+        <v>142</v>
+      </c>
+      <c r="T8" t="s">
+        <v>143</v>
+      </c>
+    </row>
+    <row r="10" spans="2:28" x14ac:dyDescent="0.25">
+      <c r="B10" s="4" t="s">
+        <v>144</v>
+      </c>
+    </row>
+    <row r="11" spans="2:28" x14ac:dyDescent="0.25">
+      <c r="F11" s="3" t="s">
+        <v>208</v>
+      </c>
+      <c r="H11" s="3" t="s">
+        <v>146</v>
+      </c>
+    </row>
+    <row r="12" spans="2:28" x14ac:dyDescent="0.25">
+      <c r="B12" s="3" t="s">
+        <v>211</v>
+      </c>
+      <c r="L12" s="3" t="s">
+        <v>155</v>
+      </c>
+      <c r="T12" s="3" t="s">
+        <v>158</v>
+      </c>
+      <c r="Z12">
+        <v>3</v>
+      </c>
+      <c r="AB12" s="3" t="s">
+        <v>162</v>
+      </c>
+    </row>
+    <row r="13" spans="2:28" x14ac:dyDescent="0.25">
+      <c r="B13" s="3" t="s">
+        <v>213</v>
+      </c>
+      <c r="L13" s="3" t="s">
+        <v>156</v>
+      </c>
+      <c r="T13" s="3" t="s">
+        <v>159</v>
+      </c>
+    </row>
+    <row r="14" spans="2:28" x14ac:dyDescent="0.25">
+      <c r="B14" s="3" t="s">
+        <v>212</v>
+      </c>
+      <c r="L14" s="3" t="s">
+        <v>157</v>
+      </c>
+      <c r="T14" s="3" t="s">
+        <v>160</v>
+      </c>
+    </row>
+    <row r="15" spans="2:28" x14ac:dyDescent="0.25">
+      <c r="B15" s="3" t="s">
+        <v>214</v>
+      </c>
+      <c r="L15" s="3" t="s">
+        <v>225</v>
+      </c>
+      <c r="T15" s="3" t="s">
+        <v>228</v>
+      </c>
+    </row>
+    <row r="17" spans="2:28" x14ac:dyDescent="0.25">
+      <c r="F17" s="3" t="s">
+        <v>145</v>
+      </c>
+      <c r="H17" s="3" t="s">
+        <v>146</v>
+      </c>
+      <c r="L17" s="3" t="s">
+        <v>155</v>
+      </c>
+      <c r="T17" s="3" t="s">
+        <v>158</v>
+      </c>
+      <c r="Z17">
+        <v>3</v>
+      </c>
+      <c r="AB17" s="3" t="s">
+        <v>163</v>
+      </c>
+    </row>
+    <row r="18" spans="2:28" x14ac:dyDescent="0.25">
+      <c r="B18" s="3" t="s">
+        <v>215</v>
+      </c>
+      <c r="L18" s="3" t="s">
+        <v>156</v>
+      </c>
+      <c r="T18" s="3" t="s">
+        <v>159</v>
+      </c>
+    </row>
+    <row r="19" spans="2:28" x14ac:dyDescent="0.25">
+      <c r="B19" s="3" t="s">
+        <v>216</v>
+      </c>
+      <c r="L19" s="3" t="s">
+        <v>157</v>
+      </c>
+      <c r="T19" s="3" t="s">
+        <v>160</v>
+      </c>
+    </row>
+    <row r="20" spans="2:28" x14ac:dyDescent="0.25">
+      <c r="B20" s="3" t="s">
+        <v>217</v>
+      </c>
+      <c r="F20" s="3"/>
+      <c r="L20" s="3" t="s">
+        <v>225</v>
+      </c>
+      <c r="T20" s="3" t="s">
+        <v>228</v>
+      </c>
+    </row>
+    <row r="21" spans="2:28" x14ac:dyDescent="0.25">
+      <c r="H21" s="3"/>
+    </row>
+    <row r="22" spans="2:28" x14ac:dyDescent="0.25">
+      <c r="F22" s="3"/>
+    </row>
+    <row r="23" spans="2:28" x14ac:dyDescent="0.25">
+      <c r="B23" s="4" t="s">
+        <v>165</v>
+      </c>
+      <c r="F23" s="3" t="s">
+        <v>166</v>
+      </c>
+      <c r="H23" s="3" t="s">
+        <v>170</v>
+      </c>
+      <c r="L23" s="3" t="s">
+        <v>172</v>
+      </c>
+      <c r="T23" s="3" t="s">
+        <v>175</v>
+      </c>
+      <c r="Z23">
+        <v>1</v>
+      </c>
+      <c r="AB23" t="s">
+        <v>177</v>
+      </c>
+    </row>
+    <row r="24" spans="2:28" x14ac:dyDescent="0.25">
+      <c r="B24" s="3" t="s">
+        <v>218</v>
+      </c>
+      <c r="F24" s="3"/>
+      <c r="L24" s="3" t="s">
+        <v>173</v>
+      </c>
+      <c r="T24" s="3" t="s">
+        <v>176</v>
+      </c>
+    </row>
+    <row r="25" spans="2:28" x14ac:dyDescent="0.25">
+      <c r="B25" s="3" t="s">
+        <v>219</v>
+      </c>
+      <c r="L25" s="3" t="s">
+        <v>157</v>
+      </c>
+      <c r="T25" s="3" t="s">
+        <v>228</v>
+      </c>
+    </row>
+    <row r="26" spans="2:28" x14ac:dyDescent="0.25">
+      <c r="B26" s="3" t="s">
+        <v>169</v>
+      </c>
+      <c r="F26" s="3"/>
+      <c r="L26" s="3" t="s">
+        <v>224</v>
+      </c>
+    </row>
+    <row r="28" spans="2:28" x14ac:dyDescent="0.25">
+      <c r="F28" s="3"/>
+    </row>
+    <row r="29" spans="2:28" x14ac:dyDescent="0.25">
+      <c r="B29" s="4" t="s">
+        <v>178</v>
+      </c>
+    </row>
+    <row r="30" spans="2:28" x14ac:dyDescent="0.25">
+      <c r="F30" s="3" t="s">
+        <v>179</v>
+      </c>
+      <c r="H30" s="3" t="s">
+        <v>184</v>
+      </c>
+      <c r="L30" s="3" t="s">
+        <v>192</v>
+      </c>
+      <c r="T30" s="3" t="s">
+        <v>193</v>
+      </c>
+      <c r="Z30">
+        <v>2</v>
+      </c>
+      <c r="AB30" s="3" t="s">
+        <v>180</v>
+      </c>
+    </row>
+    <row r="31" spans="2:28" x14ac:dyDescent="0.25">
+      <c r="B31" s="3" t="s">
+        <v>220</v>
+      </c>
+      <c r="F31" s="3"/>
+      <c r="L31" s="3" t="s">
+        <v>194</v>
+      </c>
+      <c r="T31" s="3" t="s">
+        <v>195</v>
+      </c>
+    </row>
+    <row r="32" spans="2:28" x14ac:dyDescent="0.25">
+      <c r="B32" s="3" t="s">
+        <v>221</v>
+      </c>
+      <c r="L32" s="3" t="s">
+        <v>157</v>
+      </c>
+      <c r="T32" s="3" t="s">
+        <v>228</v>
+      </c>
+    </row>
+    <row r="33" spans="2:28" x14ac:dyDescent="0.25">
+      <c r="B33" s="3" t="s">
+        <v>200</v>
+      </c>
+      <c r="F33" s="3"/>
+      <c r="T33" s="3"/>
+    </row>
+    <row r="35" spans="2:28" x14ac:dyDescent="0.25">
+      <c r="F35" s="3" t="s">
+        <v>182</v>
+      </c>
+      <c r="H35" s="3" t="s">
+        <v>183</v>
+      </c>
+      <c r="L35" s="3" t="s">
+        <v>189</v>
+      </c>
+      <c r="T35" s="3" t="s">
+        <v>188</v>
+      </c>
+      <c r="Z35">
+        <v>2</v>
+      </c>
+      <c r="AB35" t="s">
+        <v>191</v>
+      </c>
+    </row>
+    <row r="36" spans="2:28" x14ac:dyDescent="0.25">
+      <c r="B36" s="3" t="s">
+        <v>222</v>
+      </c>
+      <c r="L36" s="3" t="s">
+        <v>192</v>
+      </c>
+      <c r="T36" s="3" t="s">
+        <v>193</v>
+      </c>
+    </row>
+    <row r="37" spans="2:28" x14ac:dyDescent="0.25">
+      <c r="B37" s="3" t="s">
+        <v>186</v>
+      </c>
+      <c r="L37" s="3" t="s">
+        <v>194</v>
+      </c>
+      <c r="T37" s="3" t="s">
+        <v>195</v>
+      </c>
+    </row>
+    <row r="38" spans="2:28" x14ac:dyDescent="0.25">
+      <c r="B38" s="3" t="s">
+        <v>187</v>
+      </c>
+      <c r="L38" s="3" t="s">
+        <v>157</v>
+      </c>
+      <c r="T38" s="3" t="s">
+        <v>228</v>
+      </c>
+    </row>
+    <row r="39" spans="2:28" x14ac:dyDescent="0.25">
+      <c r="B39" s="3" t="s">
+        <v>223</v>
+      </c>
+      <c r="L39" s="3" t="s">
+        <v>224</v>
+      </c>
+      <c r="T39" s="3" t="s">
+        <v>227</v>
+      </c>
+    </row>
+    <row r="40" spans="2:28" x14ac:dyDescent="0.25">
+      <c r="L40" s="3" t="s">
+        <v>226</v>
+      </c>
+    </row>
+    <row r="44" spans="2:28" x14ac:dyDescent="0.25">
+      <c r="B44" s="3" t="s">
+        <v>201</v>
+      </c>
+    </row>
+    <row r="46" spans="2:28" x14ac:dyDescent="0.25">
+      <c r="B46" s="3" t="s">
+        <v>202</v>
+      </c>
+    </row>
+    <row r="47" spans="2:28" x14ac:dyDescent="0.25">
+      <c r="B47" s="3" t="s">
+        <v>203</v>
+      </c>
+    </row>
+    <row r="48" spans="2:28" x14ac:dyDescent="0.25">
+      <c r="B48" s="3" t="s">
+        <v>204</v>
+      </c>
+    </row>
+    <row r="50" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B50" s="3" t="s">
+        <v>205</v>
+      </c>
+    </row>
+    <row r="51" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B51" s="3" t="s">
+        <v>206</v>
+      </c>
+    </row>
+    <row r="52" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B52" s="3" t="s">
+        <v>207</v>
+      </c>
+    </row>
+  </sheetData>
+  <phoneticPr fontId="2" type="noConversion"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <dimension ref="A1"/>

</xml_diff>